<commit_message>
The latitude and longitude coordinates were backwards for Navarro's PRISM grid cells
</commit_message>
<xml_diff>
--- a/W3_LSPC_Watershed/inputs/Project_Control_Navarro.xlsx
+++ b/W3_LSPC_Watershed/inputs/Project_Control_Navarro.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E573BF99-6B83-45B2-A30F-D8308DF7E694}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDE3D457-1764-4312-B2D0-4E418F05AB7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24525" yWindow="-16395" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Flags" sheetId="10" r:id="rId1"/>
@@ -2297,10 +2297,10 @@
         <v>377987</v>
       </c>
       <c r="B2">
+        <v>38.707999999999998</v>
+      </c>
+      <c r="C2">
         <v>-123.292</v>
-      </c>
-      <c r="C2">
-        <v>38.707999999999998</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -2308,10 +2308,10 @@
         <v>377990</v>
       </c>
       <c r="B3">
+        <v>38.707999999999998</v>
+      </c>
+      <c r="C3">
         <v>-123.167</v>
-      </c>
-      <c r="C3">
-        <v>38.707999999999998</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -2319,10 +2319,10 @@
         <v>377985</v>
       </c>
       <c r="B4">
+        <v>38.707999999999998</v>
+      </c>
+      <c r="C4">
         <v>-123.375</v>
-      </c>
-      <c r="C4">
-        <v>38.707999999999998</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -2330,10 +2330,10 @@
         <v>377986</v>
       </c>
       <c r="B5">
+        <v>38.707999999999998</v>
+      </c>
+      <c r="C5">
         <v>-123.333</v>
-      </c>
-      <c r="C5">
-        <v>38.707999999999998</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -2341,10 +2341,10 @@
         <v>377988</v>
       </c>
       <c r="B6">
+        <v>38.707999999999998</v>
+      </c>
+      <c r="C6">
         <v>-123.25</v>
-      </c>
-      <c r="C6">
-        <v>38.707999999999998</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -2352,10 +2352,10 @@
         <v>377989</v>
       </c>
       <c r="B7">
+        <v>38.707999999999998</v>
+      </c>
+      <c r="C7">
         <v>-123.208</v>
-      </c>
-      <c r="C7">
-        <v>38.707999999999998</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -2363,10 +2363,10 @@
         <v>377991</v>
       </c>
       <c r="B8">
+        <v>38.707999999999998</v>
+      </c>
+      <c r="C8">
         <v>-123.125</v>
-      </c>
-      <c r="C8">
-        <v>38.707999999999998</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -2374,10 +2374,10 @@
         <v>376579</v>
       </c>
       <c r="B9">
+        <v>38.75</v>
+      </c>
+      <c r="C9">
         <v>-123.417</v>
-      </c>
-      <c r="C9">
-        <v>38.75</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -2385,10 +2385,10 @@
         <v>376582</v>
       </c>
       <c r="B10">
+        <v>38.75</v>
+      </c>
+      <c r="C10">
         <v>-123.292</v>
-      </c>
-      <c r="C10">
-        <v>38.75</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
@@ -2396,10 +2396,10 @@
         <v>376585</v>
       </c>
       <c r="B11">
+        <v>38.75</v>
+      </c>
+      <c r="C11">
         <v>-123.167</v>
-      </c>
-      <c r="C11">
-        <v>38.75</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
@@ -2407,10 +2407,10 @@
         <v>376587</v>
       </c>
       <c r="B12">
+        <v>38.75</v>
+      </c>
+      <c r="C12">
         <v>-123.083</v>
-      </c>
-      <c r="C12">
-        <v>38.75</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
@@ -2418,10 +2418,10 @@
         <v>376580</v>
       </c>
       <c r="B13">
+        <v>38.75</v>
+      </c>
+      <c r="C13">
         <v>-123.375</v>
-      </c>
-      <c r="C13">
-        <v>38.75</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -2429,10 +2429,10 @@
         <v>376581</v>
       </c>
       <c r="B14">
+        <v>38.75</v>
+      </c>
+      <c r="C14">
         <v>-123.333</v>
-      </c>
-      <c r="C14">
-        <v>38.75</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
@@ -2440,10 +2440,10 @@
         <v>376583</v>
       </c>
       <c r="B15">
+        <v>38.75</v>
+      </c>
+      <c r="C15">
         <v>-123.25</v>
-      </c>
-      <c r="C15">
-        <v>38.75</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
@@ -2451,10 +2451,10 @@
         <v>376584</v>
       </c>
       <c r="B16">
+        <v>38.75</v>
+      </c>
+      <c r="C16">
         <v>-123.208</v>
-      </c>
-      <c r="C16">
-        <v>38.75</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -2462,10 +2462,10 @@
         <v>376586</v>
       </c>
       <c r="B17">
+        <v>38.75</v>
+      </c>
+      <c r="C17">
         <v>-123.125</v>
-      </c>
-      <c r="C17">
-        <v>38.75</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
@@ -2473,10 +2473,10 @@
         <v>375174</v>
       </c>
       <c r="B18">
+        <v>38.792000000000002</v>
+      </c>
+      <c r="C18">
         <v>-123.417</v>
-      </c>
-      <c r="C18">
-        <v>38.792000000000002</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
@@ -2484,10 +2484,10 @@
         <v>375177</v>
       </c>
       <c r="B19">
+        <v>38.792000000000002</v>
+      </c>
+      <c r="C19">
         <v>-123.292</v>
-      </c>
-      <c r="C19">
-        <v>38.792000000000002</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
@@ -2495,10 +2495,10 @@
         <v>375180</v>
       </c>
       <c r="B20">
+        <v>38.792000000000002</v>
+      </c>
+      <c r="C20">
         <v>-123.167</v>
-      </c>
-      <c r="C20">
-        <v>38.792000000000002</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
@@ -2506,10 +2506,10 @@
         <v>375182</v>
       </c>
       <c r="B21">
+        <v>38.792000000000002</v>
+      </c>
+      <c r="C21">
         <v>-123.083</v>
-      </c>
-      <c r="C21">
-        <v>38.792000000000002</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
@@ -2517,10 +2517,10 @@
         <v>375173</v>
       </c>
       <c r="B22">
+        <v>38.792000000000002</v>
+      </c>
+      <c r="C22">
         <v>-123.458</v>
-      </c>
-      <c r="C22">
-        <v>38.792000000000002</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
@@ -2528,10 +2528,10 @@
         <v>375175</v>
       </c>
       <c r="B23">
+        <v>38.792000000000002</v>
+      </c>
+      <c r="C23">
         <v>-123.375</v>
-      </c>
-      <c r="C23">
-        <v>38.792000000000002</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
@@ -2539,10 +2539,10 @@
         <v>375176</v>
       </c>
       <c r="B24">
+        <v>38.792000000000002</v>
+      </c>
+      <c r="C24">
         <v>-123.333</v>
-      </c>
-      <c r="C24">
-        <v>38.792000000000002</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
@@ -2550,10 +2550,10 @@
         <v>375178</v>
       </c>
       <c r="B25">
+        <v>38.792000000000002</v>
+      </c>
+      <c r="C25">
         <v>-123.25</v>
-      </c>
-      <c r="C25">
-        <v>38.792000000000002</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
@@ -2561,10 +2561,10 @@
         <v>375179</v>
       </c>
       <c r="B26">
+        <v>38.792000000000002</v>
+      </c>
+      <c r="C26">
         <v>-123.208</v>
-      </c>
-      <c r="C26">
-        <v>38.792000000000002</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
@@ -2572,10 +2572,10 @@
         <v>375181</v>
       </c>
       <c r="B27">
+        <v>38.792000000000002</v>
+      </c>
+      <c r="C27">
         <v>-123.125</v>
-      </c>
-      <c r="C27">
-        <v>38.792000000000002</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
@@ -2583,10 +2583,10 @@
         <v>375183</v>
       </c>
       <c r="B28">
+        <v>38.792000000000002</v>
+      </c>
+      <c r="C28">
         <v>-123.042</v>
-      </c>
-      <c r="C28">
-        <v>38.792000000000002</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
@@ -2594,10 +2594,10 @@
         <v>373766</v>
       </c>
       <c r="B29">
+        <v>38.832999999999998</v>
+      </c>
+      <c r="C29">
         <v>-123.542</v>
-      </c>
-      <c r="C29">
-        <v>38.832999999999998</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
@@ -2605,10 +2605,10 @@
         <v>373769</v>
       </c>
       <c r="B30">
+        <v>38.832999999999998</v>
+      </c>
+      <c r="C30">
         <v>-123.417</v>
-      </c>
-      <c r="C30">
-        <v>38.832999999999998</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
@@ -2616,10 +2616,10 @@
         <v>373772</v>
       </c>
       <c r="B31">
+        <v>38.832999999999998</v>
+      </c>
+      <c r="C31">
         <v>-123.292</v>
-      </c>
-      <c r="C31">
-        <v>38.832999999999998</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
@@ -2627,10 +2627,10 @@
         <v>373777</v>
       </c>
       <c r="B32">
+        <v>38.832999999999998</v>
+      </c>
+      <c r="C32">
         <v>-123.083</v>
-      </c>
-      <c r="C32">
-        <v>38.832999999999998</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
@@ -2638,10 +2638,10 @@
         <v>373775</v>
       </c>
       <c r="B33">
+        <v>38.832999999999998</v>
+      </c>
+      <c r="C33">
         <v>-123.167</v>
-      </c>
-      <c r="C33">
-        <v>38.832999999999998</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
@@ -2649,10 +2649,10 @@
         <v>373767</v>
       </c>
       <c r="B34">
+        <v>38.832999999999998</v>
+      </c>
+      <c r="C34">
         <v>-123.5</v>
-      </c>
-      <c r="C34">
-        <v>38.832999999999998</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
@@ -2660,10 +2660,10 @@
         <v>373768</v>
       </c>
       <c r="B35">
+        <v>38.832999999999998</v>
+      </c>
+      <c r="C35">
         <v>-123.458</v>
-      </c>
-      <c r="C35">
-        <v>38.832999999999998</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
@@ -2671,10 +2671,10 @@
         <v>373770</v>
       </c>
       <c r="B36">
+        <v>38.832999999999998</v>
+      </c>
+      <c r="C36">
         <v>-123.375</v>
-      </c>
-      <c r="C36">
-        <v>38.832999999999998</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
@@ -2682,10 +2682,10 @@
         <v>373771</v>
       </c>
       <c r="B37">
+        <v>38.832999999999998</v>
+      </c>
+      <c r="C37">
         <v>-123.333</v>
-      </c>
-      <c r="C37">
-        <v>38.832999999999998</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
@@ -2693,10 +2693,10 @@
         <v>373773</v>
       </c>
       <c r="B38">
+        <v>38.832999999999998</v>
+      </c>
+      <c r="C38">
         <v>-123.25</v>
-      </c>
-      <c r="C38">
-        <v>38.832999999999998</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
@@ -2704,10 +2704,10 @@
         <v>373774</v>
       </c>
       <c r="B39">
+        <v>38.832999999999998</v>
+      </c>
+      <c r="C39">
         <v>-123.208</v>
-      </c>
-      <c r="C39">
-        <v>38.832999999999998</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
@@ -2715,10 +2715,10 @@
         <v>373776</v>
       </c>
       <c r="B40">
+        <v>38.832999999999998</v>
+      </c>
+      <c r="C40">
         <v>-123.125</v>
-      </c>
-      <c r="C40">
-        <v>38.832999999999998</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
@@ -2726,10 +2726,10 @@
         <v>373778</v>
       </c>
       <c r="B41">
+        <v>38.832999999999998</v>
+      </c>
+      <c r="C41">
         <v>-123.042</v>
-      </c>
-      <c r="C41">
-        <v>38.832999999999998</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
@@ -2737,10 +2737,10 @@
         <v>372361</v>
       </c>
       <c r="B42">
+        <v>38.875</v>
+      </c>
+      <c r="C42">
         <v>-123.542</v>
-      </c>
-      <c r="C42">
-        <v>38.875</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
@@ -2748,10 +2748,10 @@
         <v>372364</v>
       </c>
       <c r="B43">
+        <v>38.875</v>
+      </c>
+      <c r="C43">
         <v>-123.417</v>
-      </c>
-      <c r="C43">
-        <v>38.875</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
@@ -2759,10 +2759,10 @@
         <v>372367</v>
       </c>
       <c r="B44">
+        <v>38.875</v>
+      </c>
+      <c r="C44">
         <v>-123.292</v>
-      </c>
-      <c r="C44">
-        <v>38.875</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
@@ -2770,10 +2770,10 @@
         <v>372370</v>
       </c>
       <c r="B45">
+        <v>38.875</v>
+      </c>
+      <c r="C45">
         <v>-123.167</v>
-      </c>
-      <c r="C45">
-        <v>38.875</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
@@ -2781,10 +2781,10 @@
         <v>372372</v>
       </c>
       <c r="B46">
+        <v>38.875</v>
+      </c>
+      <c r="C46">
         <v>-123.083</v>
-      </c>
-      <c r="C46">
-        <v>38.875</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
@@ -2792,10 +2792,10 @@
         <v>372360</v>
       </c>
       <c r="B47">
+        <v>38.875</v>
+      </c>
+      <c r="C47">
         <v>-123.583</v>
-      </c>
-      <c r="C47">
-        <v>38.875</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
@@ -2803,10 +2803,10 @@
         <v>372362</v>
       </c>
       <c r="B48">
+        <v>38.875</v>
+      </c>
+      <c r="C48">
         <v>-123.5</v>
-      </c>
-      <c r="C48">
-        <v>38.875</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
@@ -2814,10 +2814,10 @@
         <v>372363</v>
       </c>
       <c r="B49">
+        <v>38.875</v>
+      </c>
+      <c r="C49">
         <v>-123.458</v>
-      </c>
-      <c r="C49">
-        <v>38.875</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
@@ -2825,10 +2825,10 @@
         <v>372365</v>
       </c>
       <c r="B50">
+        <v>38.875</v>
+      </c>
+      <c r="C50">
         <v>-123.375</v>
-      </c>
-      <c r="C50">
-        <v>38.875</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
@@ -2836,10 +2836,10 @@
         <v>372366</v>
       </c>
       <c r="B51">
+        <v>38.875</v>
+      </c>
+      <c r="C51">
         <v>-123.333</v>
-      </c>
-      <c r="C51">
-        <v>38.875</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
@@ -2847,10 +2847,10 @@
         <v>372368</v>
       </c>
       <c r="B52">
+        <v>38.875</v>
+      </c>
+      <c r="C52">
         <v>-123.25</v>
-      </c>
-      <c r="C52">
-        <v>38.875</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
@@ -2858,10 +2858,10 @@
         <v>372369</v>
       </c>
       <c r="B53">
+        <v>38.875</v>
+      </c>
+      <c r="C53">
         <v>-123.208</v>
-      </c>
-      <c r="C53">
-        <v>38.875</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
@@ -2869,10 +2869,10 @@
         <v>372371</v>
       </c>
       <c r="B54">
+        <v>38.875</v>
+      </c>
+      <c r="C54">
         <v>-123.125</v>
-      </c>
-      <c r="C54">
-        <v>38.875</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
@@ -2880,10 +2880,10 @@
         <v>372373</v>
       </c>
       <c r="B55">
+        <v>38.875</v>
+      </c>
+      <c r="C55">
         <v>-123.042</v>
-      </c>
-      <c r="C55">
-        <v>38.875</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
@@ -2891,10 +2891,10 @@
         <v>370956</v>
       </c>
       <c r="B56">
+        <v>38.917000000000002</v>
+      </c>
+      <c r="C56">
         <v>-123.542</v>
-      </c>
-      <c r="C56">
-        <v>38.917000000000002</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
@@ -2902,10 +2902,10 @@
         <v>370959</v>
       </c>
       <c r="B57">
+        <v>38.917000000000002</v>
+      </c>
+      <c r="C57">
         <v>-123.417</v>
-      </c>
-      <c r="C57">
-        <v>38.917000000000002</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
@@ -2913,10 +2913,10 @@
         <v>370962</v>
       </c>
       <c r="B58">
+        <v>38.917000000000002</v>
+      </c>
+      <c r="C58">
         <v>-123.292</v>
-      </c>
-      <c r="C58">
-        <v>38.917000000000002</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
@@ -2924,10 +2924,10 @@
         <v>370965</v>
       </c>
       <c r="B59">
+        <v>38.917000000000002</v>
+      </c>
+      <c r="C59">
         <v>-123.167</v>
-      </c>
-      <c r="C59">
-        <v>38.917000000000002</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
@@ -2935,10 +2935,10 @@
         <v>370967</v>
       </c>
       <c r="B60">
+        <v>38.917000000000002</v>
+      </c>
+      <c r="C60">
         <v>-123.083</v>
-      </c>
-      <c r="C60">
-        <v>38.917000000000002</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
@@ -2946,10 +2946,10 @@
         <v>370955</v>
       </c>
       <c r="B61">
+        <v>38.917000000000002</v>
+      </c>
+      <c r="C61">
         <v>-123.583</v>
-      </c>
-      <c r="C61">
-        <v>38.917000000000002</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
@@ -2957,10 +2957,10 @@
         <v>370957</v>
       </c>
       <c r="B62">
+        <v>38.917000000000002</v>
+      </c>
+      <c r="C62">
         <v>-123.5</v>
-      </c>
-      <c r="C62">
-        <v>38.917000000000002</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
@@ -2968,10 +2968,10 @@
         <v>370958</v>
       </c>
       <c r="B63">
+        <v>38.917000000000002</v>
+      </c>
+      <c r="C63">
         <v>-123.458</v>
-      </c>
-      <c r="C63">
-        <v>38.917000000000002</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
@@ -2979,10 +2979,10 @@
         <v>370960</v>
       </c>
       <c r="B64">
+        <v>38.917000000000002</v>
+      </c>
+      <c r="C64">
         <v>-123.375</v>
-      </c>
-      <c r="C64">
-        <v>38.917000000000002</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
@@ -2990,10 +2990,10 @@
         <v>370961</v>
       </c>
       <c r="B65">
+        <v>38.917000000000002</v>
+      </c>
+      <c r="C65">
         <v>-123.333</v>
-      </c>
-      <c r="C65">
-        <v>38.917000000000002</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.3">
@@ -3001,10 +3001,10 @@
         <v>370964</v>
       </c>
       <c r="B66">
+        <v>38.917000000000002</v>
+      </c>
+      <c r="C66">
         <v>-123.208</v>
-      </c>
-      <c r="C66">
-        <v>38.917000000000002</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.3">
@@ -3012,10 +3012,10 @@
         <v>370954</v>
       </c>
       <c r="B67">
+        <v>38.917000000000002</v>
+      </c>
+      <c r="C67">
         <v>-123.625</v>
-      </c>
-      <c r="C67">
-        <v>38.917000000000002</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
@@ -3023,10 +3023,10 @@
         <v>370963</v>
       </c>
       <c r="B68">
+        <v>38.917000000000002</v>
+      </c>
+      <c r="C68">
         <v>-123.25</v>
-      </c>
-      <c r="C68">
-        <v>38.917000000000002</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
@@ -3034,10 +3034,10 @@
         <v>370966</v>
       </c>
       <c r="B69">
+        <v>38.917000000000002</v>
+      </c>
+      <c r="C69">
         <v>-123.125</v>
-      </c>
-      <c r="C69">
-        <v>38.917000000000002</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.3">
@@ -3045,10 +3045,10 @@
         <v>370968</v>
       </c>
       <c r="B70">
+        <v>38.917000000000002</v>
+      </c>
+      <c r="C70">
         <v>-123.042</v>
-      </c>
-      <c r="C70">
-        <v>38.917000000000002</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
@@ -3056,10 +3056,10 @@
         <v>369548</v>
       </c>
       <c r="B71">
+        <v>38.957999999999998</v>
+      </c>
+      <c r="C71">
         <v>-123.667</v>
-      </c>
-      <c r="C71">
-        <v>38.957999999999998</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.3">
@@ -3067,10 +3067,10 @@
         <v>369551</v>
       </c>
       <c r="B72">
+        <v>38.957999999999998</v>
+      </c>
+      <c r="C72">
         <v>-123.542</v>
-      </c>
-      <c r="C72">
-        <v>38.957999999999998</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.3">
@@ -3078,10 +3078,10 @@
         <v>369554</v>
       </c>
       <c r="B73">
+        <v>38.957999999999998</v>
+      </c>
+      <c r="C73">
         <v>-123.417</v>
-      </c>
-      <c r="C73">
-        <v>38.957999999999998</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.3">
@@ -3089,10 +3089,10 @@
         <v>369557</v>
       </c>
       <c r="B74">
+        <v>38.957999999999998</v>
+      </c>
+      <c r="C74">
         <v>-123.292</v>
-      </c>
-      <c r="C74">
-        <v>38.957999999999998</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.3">
@@ -3100,10 +3100,10 @@
         <v>369562</v>
       </c>
       <c r="B75">
+        <v>38.957999999999998</v>
+      </c>
+      <c r="C75">
         <v>-123.083</v>
-      </c>
-      <c r="C75">
-        <v>38.957999999999998</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.3">
@@ -3111,10 +3111,10 @@
         <v>369560</v>
       </c>
       <c r="B76">
+        <v>38.957999999999998</v>
+      </c>
+      <c r="C76">
         <v>-123.167</v>
-      </c>
-      <c r="C76">
-        <v>38.957999999999998</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.3">
@@ -3122,10 +3122,10 @@
         <v>369550</v>
       </c>
       <c r="B77">
+        <v>38.957999999999998</v>
+      </c>
+      <c r="C77">
         <v>-123.583</v>
-      </c>
-      <c r="C77">
-        <v>38.957999999999998</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.3">
@@ -3133,10 +3133,10 @@
         <v>369549</v>
       </c>
       <c r="B78">
+        <v>38.957999999999998</v>
+      </c>
+      <c r="C78">
         <v>-123.625</v>
-      </c>
-      <c r="C78">
-        <v>38.957999999999998</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.3">
@@ -3144,10 +3144,10 @@
         <v>369552</v>
       </c>
       <c r="B79">
+        <v>38.957999999999998</v>
+      </c>
+      <c r="C79">
         <v>-123.5</v>
-      </c>
-      <c r="C79">
-        <v>38.957999999999998</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.3">
@@ -3155,10 +3155,10 @@
         <v>369553</v>
       </c>
       <c r="B80">
+        <v>38.957999999999998</v>
+      </c>
+      <c r="C80">
         <v>-123.458</v>
-      </c>
-      <c r="C80">
-        <v>38.957999999999998</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.3">
@@ -3166,10 +3166,10 @@
         <v>369555</v>
       </c>
       <c r="B81">
+        <v>38.957999999999998</v>
+      </c>
+      <c r="C81">
         <v>-123.375</v>
-      </c>
-      <c r="C81">
-        <v>38.957999999999998</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.3">
@@ -3177,10 +3177,10 @@
         <v>369556</v>
       </c>
       <c r="B82">
+        <v>38.957999999999998</v>
+      </c>
+      <c r="C82">
         <v>-123.333</v>
-      </c>
-      <c r="C82">
-        <v>38.957999999999998</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.3">
@@ -3188,10 +3188,10 @@
         <v>369558</v>
       </c>
       <c r="B83">
+        <v>38.957999999999998</v>
+      </c>
+      <c r="C83">
         <v>-123.25</v>
-      </c>
-      <c r="C83">
-        <v>38.957999999999998</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.3">
@@ -3199,10 +3199,10 @@
         <v>369559</v>
       </c>
       <c r="B84">
+        <v>38.957999999999998</v>
+      </c>
+      <c r="C84">
         <v>-123.208</v>
-      </c>
-      <c r="C84">
-        <v>38.957999999999998</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.3">
@@ -3210,10 +3210,10 @@
         <v>369561</v>
       </c>
       <c r="B85">
+        <v>38.957999999999998</v>
+      </c>
+      <c r="C85">
         <v>-123.125</v>
-      </c>
-      <c r="C85">
-        <v>38.957999999999998</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.3">
@@ -3221,10 +3221,10 @@
         <v>369563</v>
       </c>
       <c r="B86">
+        <v>38.957999999999998</v>
+      </c>
+      <c r="C86">
         <v>-123.042</v>
-      </c>
-      <c r="C86">
-        <v>38.957999999999998</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.3">
@@ -3232,10 +3232,10 @@
         <v>368143</v>
       </c>
       <c r="B87">
+        <v>39</v>
+      </c>
+      <c r="C87">
         <v>-123.667</v>
-      </c>
-      <c r="C87">
-        <v>39</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.3">
@@ -3243,10 +3243,10 @@
         <v>368146</v>
       </c>
       <c r="B88">
+        <v>39</v>
+      </c>
+      <c r="C88">
         <v>-123.542</v>
-      </c>
-      <c r="C88">
-        <v>39</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.3">
@@ -3254,10 +3254,10 @@
         <v>368149</v>
       </c>
       <c r="B89">
+        <v>39</v>
+      </c>
+      <c r="C89">
         <v>-123.417</v>
-      </c>
-      <c r="C89">
-        <v>39</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.3">
@@ -3265,10 +3265,10 @@
         <v>368155</v>
       </c>
       <c r="B90">
+        <v>39</v>
+      </c>
+      <c r="C90">
         <v>-123.167</v>
-      </c>
-      <c r="C90">
-        <v>39</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.3">
@@ -3276,10 +3276,10 @@
         <v>368157</v>
       </c>
       <c r="B91">
+        <v>39</v>
+      </c>
+      <c r="C91">
         <v>-123.083</v>
-      </c>
-      <c r="C91">
-        <v>39</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.3">
@@ -3287,10 +3287,10 @@
         <v>368152</v>
       </c>
       <c r="B92">
+        <v>39</v>
+      </c>
+      <c r="C92">
         <v>-123.292</v>
-      </c>
-      <c r="C92">
-        <v>39</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.3">
@@ -3298,10 +3298,10 @@
         <v>368142</v>
       </c>
       <c r="B93">
+        <v>39</v>
+      </c>
+      <c r="C93">
         <v>-123.708</v>
-      </c>
-      <c r="C93">
-        <v>39</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.3">
@@ -3309,10 +3309,10 @@
         <v>368145</v>
       </c>
       <c r="B94">
+        <v>39</v>
+      </c>
+      <c r="C94">
         <v>-123.583</v>
-      </c>
-      <c r="C94">
-        <v>39</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.3">
@@ -3320,10 +3320,10 @@
         <v>368148</v>
       </c>
       <c r="B95">
+        <v>39</v>
+      </c>
+      <c r="C95">
         <v>-123.458</v>
-      </c>
-      <c r="C95">
-        <v>39</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.3">
@@ -3331,10 +3331,10 @@
         <v>368151</v>
       </c>
       <c r="B96">
+        <v>39</v>
+      </c>
+      <c r="C96">
         <v>-123.333</v>
-      </c>
-      <c r="C96">
-        <v>39</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.3">
@@ -3342,10 +3342,10 @@
         <v>368154</v>
       </c>
       <c r="B97">
+        <v>39</v>
+      </c>
+      <c r="C97">
         <v>-123.208</v>
-      </c>
-      <c r="C97">
-        <v>39</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.3">
@@ -3353,10 +3353,10 @@
         <v>368156</v>
       </c>
       <c r="B98">
+        <v>39</v>
+      </c>
+      <c r="C98">
         <v>-123.125</v>
-      </c>
-      <c r="C98">
-        <v>39</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.3">
@@ -3364,10 +3364,10 @@
         <v>368144</v>
       </c>
       <c r="B99">
+        <v>39</v>
+      </c>
+      <c r="C99">
         <v>-123.625</v>
-      </c>
-      <c r="C99">
-        <v>39</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.3">
@@ -3375,10 +3375,10 @@
         <v>368147</v>
       </c>
       <c r="B100">
+        <v>39</v>
+      </c>
+      <c r="C100">
         <v>-123.5</v>
-      </c>
-      <c r="C100">
-        <v>39</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.3">
@@ -3386,10 +3386,10 @@
         <v>368150</v>
       </c>
       <c r="B101">
+        <v>39</v>
+      </c>
+      <c r="C101">
         <v>-123.375</v>
-      </c>
-      <c r="C101">
-        <v>39</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.3">
@@ -3397,10 +3397,10 @@
         <v>368153</v>
       </c>
       <c r="B102">
+        <v>39</v>
+      </c>
+      <c r="C102">
         <v>-123.25</v>
-      </c>
-      <c r="C102">
-        <v>39</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.3">
@@ -3408,10 +3408,10 @@
         <v>366738</v>
       </c>
       <c r="B103">
+        <v>39.042000000000002</v>
+      </c>
+      <c r="C103">
         <v>-123.667</v>
-      </c>
-      <c r="C103">
-        <v>39.042000000000002</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.3">
@@ -3419,10 +3419,10 @@
         <v>366741</v>
       </c>
       <c r="B104">
+        <v>39.042000000000002</v>
+      </c>
+      <c r="C104">
         <v>-123.542</v>
-      </c>
-      <c r="C104">
-        <v>39.042000000000002</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.3">
@@ -3430,10 +3430,10 @@
         <v>366744</v>
       </c>
       <c r="B105">
+        <v>39.042000000000002</v>
+      </c>
+      <c r="C105">
         <v>-123.417</v>
-      </c>
-      <c r="C105">
-        <v>39.042000000000002</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.3">
@@ -3441,10 +3441,10 @@
         <v>366750</v>
       </c>
       <c r="B106">
+        <v>39.042000000000002</v>
+      </c>
+      <c r="C106">
         <v>-123.167</v>
-      </c>
-      <c r="C106">
-        <v>39.042000000000002</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.3">
@@ -3452,10 +3452,10 @@
         <v>366752</v>
       </c>
       <c r="B107">
+        <v>39.042000000000002</v>
+      </c>
+      <c r="C107">
         <v>-123.083</v>
-      </c>
-      <c r="C107">
-        <v>39.042000000000002</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.3">
@@ -3463,10 +3463,10 @@
         <v>366747</v>
       </c>
       <c r="B108">
+        <v>39.042000000000002</v>
+      </c>
+      <c r="C108">
         <v>-123.292</v>
-      </c>
-      <c r="C108">
-        <v>39.042000000000002</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.3">
@@ -3474,10 +3474,10 @@
         <v>366740</v>
       </c>
       <c r="B109">
+        <v>39.042000000000002</v>
+      </c>
+      <c r="C109">
         <v>-123.583</v>
-      </c>
-      <c r="C109">
-        <v>39.042000000000002</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.3">
@@ -3485,10 +3485,10 @@
         <v>366742</v>
       </c>
       <c r="B110">
+        <v>39.042000000000002</v>
+      </c>
+      <c r="C110">
         <v>-123.5</v>
-      </c>
-      <c r="C110">
-        <v>39.042000000000002</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.3">
@@ -3496,10 +3496,10 @@
         <v>366743</v>
       </c>
       <c r="B111">
+        <v>39.042000000000002</v>
+      </c>
+      <c r="C111">
         <v>-123.458</v>
-      </c>
-      <c r="C111">
-        <v>39.042000000000002</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.3">
@@ -3507,10 +3507,10 @@
         <v>366746</v>
       </c>
       <c r="B112">
+        <v>39.042000000000002</v>
+      </c>
+      <c r="C112">
         <v>-123.333</v>
-      </c>
-      <c r="C112">
-        <v>39.042000000000002</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.3">
@@ -3518,10 +3518,10 @@
         <v>366749</v>
       </c>
       <c r="B113">
+        <v>39.042000000000002</v>
+      </c>
+      <c r="C113">
         <v>-123.208</v>
-      </c>
-      <c r="C113">
-        <v>39.042000000000002</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.3">
@@ -3529,10 +3529,10 @@
         <v>366739</v>
       </c>
       <c r="B114">
+        <v>39.042000000000002</v>
+      </c>
+      <c r="C114">
         <v>-123.625</v>
-      </c>
-      <c r="C114">
-        <v>39.042000000000002</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.3">
@@ -3540,10 +3540,10 @@
         <v>366745</v>
       </c>
       <c r="B115">
+        <v>39.042000000000002</v>
+      </c>
+      <c r="C115">
         <v>-123.375</v>
-      </c>
-      <c r="C115">
-        <v>39.042000000000002</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.3">
@@ -3551,10 +3551,10 @@
         <v>366748</v>
       </c>
       <c r="B116">
+        <v>39.042000000000002</v>
+      </c>
+      <c r="C116">
         <v>-123.25</v>
-      </c>
-      <c r="C116">
-        <v>39.042000000000002</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.3">
@@ -3562,10 +3562,10 @@
         <v>366751</v>
       </c>
       <c r="B117">
+        <v>39.042000000000002</v>
+      </c>
+      <c r="C117">
         <v>-123.125</v>
-      </c>
-      <c r="C117">
-        <v>39.042000000000002</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.3">
@@ -3573,10 +3573,10 @@
         <v>366737</v>
       </c>
       <c r="B118">
+        <v>39.042000000000002</v>
+      </c>
+      <c r="C118">
         <v>-123.708</v>
-      </c>
-      <c r="C118">
-        <v>39.042000000000002</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.3">
@@ -3584,10 +3584,10 @@
         <v>365333</v>
       </c>
       <c r="B119">
+        <v>39.082999999999998</v>
+      </c>
+      <c r="C119">
         <v>-123.667</v>
-      </c>
-      <c r="C119">
-        <v>39.082999999999998</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.3">
@@ -3595,10 +3595,10 @@
         <v>365336</v>
       </c>
       <c r="B120">
+        <v>39.082999999999998</v>
+      </c>
+      <c r="C120">
         <v>-123.542</v>
-      </c>
-      <c r="C120">
-        <v>39.082999999999998</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.3">
@@ -3606,10 +3606,10 @@
         <v>365342</v>
       </c>
       <c r="B121">
+        <v>39.082999999999998</v>
+      </c>
+      <c r="C121">
         <v>-123.292</v>
-      </c>
-      <c r="C121">
-        <v>39.082999999999998</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.3">
@@ -3617,10 +3617,10 @@
         <v>365345</v>
       </c>
       <c r="B122">
+        <v>39.082999999999998</v>
+      </c>
+      <c r="C122">
         <v>-123.167</v>
-      </c>
-      <c r="C122">
-        <v>39.082999999999998</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.3">
@@ -3628,10 +3628,10 @@
         <v>365339</v>
       </c>
       <c r="B123">
+        <v>39.082999999999998</v>
+      </c>
+      <c r="C123">
         <v>-123.417</v>
-      </c>
-      <c r="C123">
-        <v>39.082999999999998</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.3">
@@ -3639,10 +3639,10 @@
         <v>365335</v>
       </c>
       <c r="B124">
+        <v>39.082999999999998</v>
+      </c>
+      <c r="C124">
         <v>-123.583</v>
-      </c>
-      <c r="C124">
-        <v>39.082999999999998</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.3">
@@ -3650,10 +3650,10 @@
         <v>365334</v>
       </c>
       <c r="B125">
+        <v>39.082999999999998</v>
+      </c>
+      <c r="C125">
         <v>-123.625</v>
-      </c>
-      <c r="C125">
-        <v>39.082999999999998</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.3">
@@ -3661,10 +3661,10 @@
         <v>365337</v>
       </c>
       <c r="B126">
+        <v>39.082999999999998</v>
+      </c>
+      <c r="C126">
         <v>-123.5</v>
-      </c>
-      <c r="C126">
-        <v>39.082999999999998</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.3">
@@ -3672,10 +3672,10 @@
         <v>365338</v>
       </c>
       <c r="B127">
+        <v>39.082999999999998</v>
+      </c>
+      <c r="C127">
         <v>-123.458</v>
-      </c>
-      <c r="C127">
-        <v>39.082999999999998</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.3">
@@ -3683,10 +3683,10 @@
         <v>365341</v>
       </c>
       <c r="B128">
+        <v>39.082999999999998</v>
+      </c>
+      <c r="C128">
         <v>-123.333</v>
-      </c>
-      <c r="C128">
-        <v>39.082999999999998</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.3">
@@ -3694,10 +3694,10 @@
         <v>365344</v>
       </c>
       <c r="B129">
+        <v>39.082999999999998</v>
+      </c>
+      <c r="C129">
         <v>-123.208</v>
-      </c>
-      <c r="C129">
-        <v>39.082999999999998</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.3">
@@ -3705,10 +3705,10 @@
         <v>365340</v>
       </c>
       <c r="B130">
+        <v>39.082999999999998</v>
+      </c>
+      <c r="C130">
         <v>-123.375</v>
-      </c>
-      <c r="C130">
-        <v>39.082999999999998</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.3">
@@ -3716,10 +3716,10 @@
         <v>365343</v>
       </c>
       <c r="B131">
+        <v>39.082999999999998</v>
+      </c>
+      <c r="C131">
         <v>-123.25</v>
-      </c>
-      <c r="C131">
-        <v>39.082999999999998</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.3">
@@ -3727,10 +3727,10 @@
         <v>365346</v>
       </c>
       <c r="B132">
+        <v>39.082999999999998</v>
+      </c>
+      <c r="C132">
         <v>-123.125</v>
-      </c>
-      <c r="C132">
-        <v>39.082999999999998</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.3">
@@ -3738,10 +3738,10 @@
         <v>365332</v>
       </c>
       <c r="B133">
+        <v>39.082999999999998</v>
+      </c>
+      <c r="C133">
         <v>-123.708</v>
-      </c>
-      <c r="C133">
-        <v>39.082999999999998</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.3">
@@ -3749,10 +3749,10 @@
         <v>363928</v>
       </c>
       <c r="B134">
+        <v>39.125</v>
+      </c>
+      <c r="C134">
         <v>-123.667</v>
-      </c>
-      <c r="C134">
-        <v>39.125</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.3">
@@ -3760,10 +3760,10 @@
         <v>363931</v>
       </c>
       <c r="B135">
+        <v>39.125</v>
+      </c>
+      <c r="C135">
         <v>-123.542</v>
-      </c>
-      <c r="C135">
-        <v>39.125</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.3">
@@ -3771,10 +3771,10 @@
         <v>363934</v>
       </c>
       <c r="B136">
+        <v>39.125</v>
+      </c>
+      <c r="C136">
         <v>-123.417</v>
-      </c>
-      <c r="C136">
-        <v>39.125</v>
       </c>
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.3">
@@ -3782,10 +3782,10 @@
         <v>363937</v>
       </c>
       <c r="B137">
+        <v>39.125</v>
+      </c>
+      <c r="C137">
         <v>-123.292</v>
-      </c>
-      <c r="C137">
-        <v>39.125</v>
       </c>
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.3">
@@ -3793,10 +3793,10 @@
         <v>363940</v>
       </c>
       <c r="B138">
+        <v>39.125</v>
+      </c>
+      <c r="C138">
         <v>-123.167</v>
-      </c>
-      <c r="C138">
-        <v>39.125</v>
       </c>
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.3">
@@ -3804,10 +3804,10 @@
         <v>363926</v>
       </c>
       <c r="B139">
+        <v>39.125</v>
+      </c>
+      <c r="C139">
         <v>-123.75</v>
-      </c>
-      <c r="C139">
-        <v>39.125</v>
       </c>
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.3">
@@ -3815,10 +3815,10 @@
         <v>363927</v>
       </c>
       <c r="B140">
+        <v>39.125</v>
+      </c>
+      <c r="C140">
         <v>-123.708</v>
-      </c>
-      <c r="C140">
-        <v>39.125</v>
       </c>
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.3">
@@ -3826,10 +3826,10 @@
         <v>363930</v>
       </c>
       <c r="B141">
+        <v>39.125</v>
+      </c>
+      <c r="C141">
         <v>-123.583</v>
-      </c>
-      <c r="C141">
-        <v>39.125</v>
       </c>
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.3">
@@ -3837,10 +3837,10 @@
         <v>363932</v>
       </c>
       <c r="B142">
+        <v>39.125</v>
+      </c>
+      <c r="C142">
         <v>-123.5</v>
-      </c>
-      <c r="C142">
-        <v>39.125</v>
       </c>
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.3">
@@ -3848,10 +3848,10 @@
         <v>363933</v>
       </c>
       <c r="B143">
+        <v>39.125</v>
+      </c>
+      <c r="C143">
         <v>-123.458</v>
-      </c>
-      <c r="C143">
-        <v>39.125</v>
       </c>
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.3">
@@ -3859,10 +3859,10 @@
         <v>363936</v>
       </c>
       <c r="B144">
+        <v>39.125</v>
+      </c>
+      <c r="C144">
         <v>-123.333</v>
-      </c>
-      <c r="C144">
-        <v>39.125</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.3">
@@ -3870,10 +3870,10 @@
         <v>363939</v>
       </c>
       <c r="B145">
+        <v>39.125</v>
+      </c>
+      <c r="C145">
         <v>-123.208</v>
-      </c>
-      <c r="C145">
-        <v>39.125</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.3">
@@ -3881,10 +3881,10 @@
         <v>363929</v>
       </c>
       <c r="B146">
+        <v>39.125</v>
+      </c>
+      <c r="C146">
         <v>-123.625</v>
-      </c>
-      <c r="C146">
-        <v>39.125</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.3">
@@ -3892,10 +3892,10 @@
         <v>363935</v>
       </c>
       <c r="B147">
+        <v>39.125</v>
+      </c>
+      <c r="C147">
         <v>-123.375</v>
-      </c>
-      <c r="C147">
-        <v>39.125</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.3">
@@ -3903,10 +3903,10 @@
         <v>363938</v>
       </c>
       <c r="B148">
+        <v>39.125</v>
+      </c>
+      <c r="C148">
         <v>-123.25</v>
-      </c>
-      <c r="C148">
-        <v>39.125</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.3">
@@ -3914,10 +3914,10 @@
         <v>363941</v>
       </c>
       <c r="B149">
+        <v>39.125</v>
+      </c>
+      <c r="C149">
         <v>-123.125</v>
-      </c>
-      <c r="C149">
-        <v>39.125</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.3">
@@ -3925,10 +3925,10 @@
         <v>362523</v>
       </c>
       <c r="B150">
+        <v>39.167000000000002</v>
+      </c>
+      <c r="C150">
         <v>-123.667</v>
-      </c>
-      <c r="C150">
-        <v>39.167000000000002</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.3">
@@ -3936,10 +3936,10 @@
         <v>362526</v>
       </c>
       <c r="B151">
+        <v>39.167000000000002</v>
+      </c>
+      <c r="C151">
         <v>-123.542</v>
-      </c>
-      <c r="C151">
-        <v>39.167000000000002</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.3">
@@ -3947,10 +3947,10 @@
         <v>362529</v>
       </c>
       <c r="B152">
+        <v>39.167000000000002</v>
+      </c>
+      <c r="C152">
         <v>-123.417</v>
-      </c>
-      <c r="C152">
-        <v>39.167000000000002</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.3">
@@ -3958,10 +3958,10 @@
         <v>362532</v>
       </c>
       <c r="B153">
+        <v>39.167000000000002</v>
+      </c>
+      <c r="C153">
         <v>-123.292</v>
-      </c>
-      <c r="C153">
-        <v>39.167000000000002</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.3">
@@ -3969,10 +3969,10 @@
         <v>362535</v>
       </c>
       <c r="B154">
+        <v>39.167000000000002</v>
+      </c>
+      <c r="C154">
         <v>-123.167</v>
-      </c>
-      <c r="C154">
-        <v>39.167000000000002</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.3">
@@ -3980,10 +3980,10 @@
         <v>362522</v>
       </c>
       <c r="B155">
+        <v>39.167000000000002</v>
+      </c>
+      <c r="C155">
         <v>-123.708</v>
-      </c>
-      <c r="C155">
-        <v>39.167000000000002</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.3">
@@ -3991,10 +3991,10 @@
         <v>362524</v>
       </c>
       <c r="B156">
+        <v>39.167000000000002</v>
+      </c>
+      <c r="C156">
         <v>-123.625</v>
-      </c>
-      <c r="C156">
-        <v>39.167000000000002</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.3">
@@ -4002,10 +4002,10 @@
         <v>362525</v>
       </c>
       <c r="B157">
+        <v>39.167000000000002</v>
+      </c>
+      <c r="C157">
         <v>-123.583</v>
-      </c>
-      <c r="C157">
-        <v>39.167000000000002</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.3">
@@ -4013,10 +4013,10 @@
         <v>362528</v>
       </c>
       <c r="B158">
+        <v>39.167000000000002</v>
+      </c>
+      <c r="C158">
         <v>-123.458</v>
-      </c>
-      <c r="C158">
-        <v>39.167000000000002</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.3">
@@ -4024,10 +4024,10 @@
         <v>362531</v>
       </c>
       <c r="B159">
+        <v>39.167000000000002</v>
+      </c>
+      <c r="C159">
         <v>-123.333</v>
-      </c>
-      <c r="C159">
-        <v>39.167000000000002</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.3">
@@ -4035,10 +4035,10 @@
         <v>362534</v>
       </c>
       <c r="B160">
+        <v>39.167000000000002</v>
+      </c>
+      <c r="C160">
         <v>-123.208</v>
-      </c>
-      <c r="C160">
-        <v>39.167000000000002</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.3">
@@ -4046,10 +4046,10 @@
         <v>362527</v>
       </c>
       <c r="B161">
+        <v>39.167000000000002</v>
+      </c>
+      <c r="C161">
         <v>-123.5</v>
-      </c>
-      <c r="C161">
-        <v>39.167000000000002</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.3">
@@ -4057,10 +4057,10 @@
         <v>362530</v>
       </c>
       <c r="B162">
+        <v>39.167000000000002</v>
+      </c>
+      <c r="C162">
         <v>-123.375</v>
-      </c>
-      <c r="C162">
-        <v>39.167000000000002</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.3">
@@ -4068,10 +4068,10 @@
         <v>362533</v>
       </c>
       <c r="B163">
+        <v>39.167000000000002</v>
+      </c>
+      <c r="C163">
         <v>-123.25</v>
-      </c>
-      <c r="C163">
-        <v>39.167000000000002</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.3">
@@ -4079,10 +4079,10 @@
         <v>362521</v>
       </c>
       <c r="B164">
+        <v>39.167000000000002</v>
+      </c>
+      <c r="C164">
         <v>-123.75</v>
-      </c>
-      <c r="C164">
-        <v>39.167000000000002</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.3">
@@ -4090,10 +4090,10 @@
         <v>361127</v>
       </c>
       <c r="B165">
+        <v>39.207999999999998</v>
+      </c>
+      <c r="C165">
         <v>-123.292</v>
-      </c>
-      <c r="C165">
-        <v>39.207999999999998</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.3">
@@ -4101,10 +4101,10 @@
         <v>361130</v>
       </c>
       <c r="B166">
+        <v>39.207999999999998</v>
+      </c>
+      <c r="C166">
         <v>-123.167</v>
-      </c>
-      <c r="C166">
-        <v>39.207999999999998</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.3">
@@ -4112,10 +4112,10 @@
         <v>361118</v>
       </c>
       <c r="B167">
+        <v>39.207999999999998</v>
+      </c>
+      <c r="C167">
         <v>-123.667</v>
-      </c>
-      <c r="C167">
-        <v>39.207999999999998</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.3">
@@ -4123,10 +4123,10 @@
         <v>361121</v>
       </c>
       <c r="B168">
+        <v>39.207999999999998</v>
+      </c>
+      <c r="C168">
         <v>-123.542</v>
-      </c>
-      <c r="C168">
-        <v>39.207999999999998</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.3">
@@ -4134,10 +4134,10 @@
         <v>361124</v>
       </c>
       <c r="B169">
+        <v>39.207999999999998</v>
+      </c>
+      <c r="C169">
         <v>-123.417</v>
-      </c>
-      <c r="C169">
-        <v>39.207999999999998</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.3">
@@ -4145,10 +4145,10 @@
         <v>361115</v>
       </c>
       <c r="B170">
+        <v>39.207999999999998</v>
+      </c>
+      <c r="C170">
         <v>-123.792</v>
-      </c>
-      <c r="C170">
-        <v>39.207999999999998</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.3">
@@ -4156,10 +4156,10 @@
         <v>361120</v>
       </c>
       <c r="B171">
+        <v>39.207999999999998</v>
+      </c>
+      <c r="C171">
         <v>-123.583</v>
-      </c>
-      <c r="C171">
-        <v>39.207999999999998</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.3">
@@ -4167,10 +4167,10 @@
         <v>361117</v>
       </c>
       <c r="B172">
+        <v>39.207999999999998</v>
+      </c>
+      <c r="C172">
         <v>-123.708</v>
-      </c>
-      <c r="C172">
-        <v>39.207999999999998</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.3">
@@ -4178,10 +4178,10 @@
         <v>361116</v>
       </c>
       <c r="B173">
+        <v>39.207999999999998</v>
+      </c>
+      <c r="C173">
         <v>-123.75</v>
-      </c>
-      <c r="C173">
-        <v>39.207999999999998</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.3">
@@ -4189,10 +4189,10 @@
         <v>361119</v>
       </c>
       <c r="B174">
+        <v>39.207999999999998</v>
+      </c>
+      <c r="C174">
         <v>-123.625</v>
-      </c>
-      <c r="C174">
-        <v>39.207999999999998</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.3">
@@ -4200,10 +4200,10 @@
         <v>361122</v>
       </c>
       <c r="B175">
+        <v>39.207999999999998</v>
+      </c>
+      <c r="C175">
         <v>-123.5</v>
-      </c>
-      <c r="C175">
-        <v>39.207999999999998</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.3">
@@ -4211,10 +4211,10 @@
         <v>361123</v>
       </c>
       <c r="B176">
+        <v>39.207999999999998</v>
+      </c>
+      <c r="C176">
         <v>-123.458</v>
-      </c>
-      <c r="C176">
-        <v>39.207999999999998</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.3">
@@ -4222,10 +4222,10 @@
         <v>361125</v>
       </c>
       <c r="B177">
+        <v>39.207999999999998</v>
+      </c>
+      <c r="C177">
         <v>-123.375</v>
-      </c>
-      <c r="C177">
-        <v>39.207999999999998</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.3">
@@ -4233,10 +4233,10 @@
         <v>361126</v>
       </c>
       <c r="B178">
+        <v>39.207999999999998</v>
+      </c>
+      <c r="C178">
         <v>-123.333</v>
-      </c>
-      <c r="C178">
-        <v>39.207999999999998</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.3">
@@ -4244,10 +4244,10 @@
         <v>361128</v>
       </c>
       <c r="B179">
+        <v>39.207999999999998</v>
+      </c>
+      <c r="C179">
         <v>-123.25</v>
-      </c>
-      <c r="C179">
-        <v>39.207999999999998</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.3">
@@ -4255,10 +4255,10 @@
         <v>361129</v>
       </c>
       <c r="B180">
+        <v>39.207999999999998</v>
+      </c>
+      <c r="C180">
         <v>-123.208</v>
-      </c>
-      <c r="C180">
-        <v>39.207999999999998</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.3">
@@ -4266,10 +4266,10 @@
         <v>359713</v>
       </c>
       <c r="B181">
+        <v>39.25</v>
+      </c>
+      <c r="C181">
         <v>-123.667</v>
-      </c>
-      <c r="C181">
-        <v>39.25</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.3">
@@ -4277,10 +4277,10 @@
         <v>359716</v>
       </c>
       <c r="B182">
+        <v>39.25</v>
+      </c>
+      <c r="C182">
         <v>-123.542</v>
-      </c>
-      <c r="C182">
-        <v>39.25</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.3">
@@ -4288,10 +4288,10 @@
         <v>359719</v>
       </c>
       <c r="B183">
+        <v>39.25</v>
+      </c>
+      <c r="C183">
         <v>-123.417</v>
-      </c>
-      <c r="C183">
-        <v>39.25</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.3">
@@ -4299,10 +4299,10 @@
         <v>359722</v>
       </c>
       <c r="B184">
+        <v>39.25</v>
+      </c>
+      <c r="C184">
         <v>-123.292</v>
-      </c>
-      <c r="C184">
-        <v>39.25</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.3">
@@ -4310,10 +4310,10 @@
         <v>359711</v>
       </c>
       <c r="B185">
+        <v>39.25</v>
+      </c>
+      <c r="C185">
         <v>-123.75</v>
-      </c>
-      <c r="C185">
-        <v>39.25</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.3">
@@ -4321,10 +4321,10 @@
         <v>359712</v>
       </c>
       <c r="B186">
+        <v>39.25</v>
+      </c>
+      <c r="C186">
         <v>-123.708</v>
-      </c>
-      <c r="C186">
-        <v>39.25</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.3">
@@ -4332,10 +4332,10 @@
         <v>359714</v>
       </c>
       <c r="B187">
+        <v>39.25</v>
+      </c>
+      <c r="C187">
         <v>-123.625</v>
-      </c>
-      <c r="C187">
-        <v>39.25</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.3">
@@ -4343,10 +4343,10 @@
         <v>359715</v>
       </c>
       <c r="B188">
+        <v>39.25</v>
+      </c>
+      <c r="C188">
         <v>-123.583</v>
-      </c>
-      <c r="C188">
-        <v>39.25</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.3">
@@ -4354,10 +4354,10 @@
         <v>359717</v>
       </c>
       <c r="B189">
+        <v>39.25</v>
+      </c>
+      <c r="C189">
         <v>-123.5</v>
-      </c>
-      <c r="C189">
-        <v>39.25</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.3">
@@ -4365,10 +4365,10 @@
         <v>359718</v>
       </c>
       <c r="B190">
+        <v>39.25</v>
+      </c>
+      <c r="C190">
         <v>-123.458</v>
-      </c>
-      <c r="C190">
-        <v>39.25</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.3">
@@ -4376,10 +4376,10 @@
         <v>359720</v>
       </c>
       <c r="B191">
+        <v>39.25</v>
+      </c>
+      <c r="C191">
         <v>-123.375</v>
-      </c>
-      <c r="C191">
-        <v>39.25</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.3">
@@ -4387,10 +4387,10 @@
         <v>359721</v>
       </c>
       <c r="B192">
+        <v>39.25</v>
+      </c>
+      <c r="C192">
         <v>-123.333</v>
-      </c>
-      <c r="C192">
-        <v>39.25</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.3">
@@ -4398,10 +4398,10 @@
         <v>359723</v>
       </c>
       <c r="B193">
+        <v>39.25</v>
+      </c>
+      <c r="C193">
         <v>-123.25</v>
-      </c>
-      <c r="C193">
-        <v>39.25</v>
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.3">
@@ -4409,10 +4409,10 @@
         <v>359724</v>
       </c>
       <c r="B194">
+        <v>39.25</v>
+      </c>
+      <c r="C194">
         <v>-123.208</v>
-      </c>
-      <c r="C194">
-        <v>39.25</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.3">
@@ -4420,10 +4420,10 @@
         <v>359710</v>
       </c>
       <c r="B195">
+        <v>39.25</v>
+      </c>
+      <c r="C195">
         <v>-123.792</v>
-      </c>
-      <c r="C195">
-        <v>39.25</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.3">
@@ -4431,10 +4431,10 @@
         <v>358304</v>
       </c>
       <c r="B196">
+        <v>39.292000000000002</v>
+      </c>
+      <c r="C196">
         <v>-123.833</v>
-      </c>
-      <c r="C196">
-        <v>39.292000000000002</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.3">
@@ -4442,10 +4442,10 @@
         <v>358308</v>
       </c>
       <c r="B197">
+        <v>39.292000000000002</v>
+      </c>
+      <c r="C197">
         <v>-123.667</v>
-      </c>
-      <c r="C197">
-        <v>39.292000000000002</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.3">
@@ -4453,10 +4453,10 @@
         <v>358311</v>
       </c>
       <c r="B198">
+        <v>39.292000000000002</v>
+      </c>
+      <c r="C198">
         <v>-123.542</v>
-      </c>
-      <c r="C198">
-        <v>39.292000000000002</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.3">
@@ -4464,10 +4464,10 @@
         <v>358314</v>
       </c>
       <c r="B199">
+        <v>39.292000000000002</v>
+      </c>
+      <c r="C199">
         <v>-123.417</v>
-      </c>
-      <c r="C199">
-        <v>39.292000000000002</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.3">
@@ -4475,10 +4475,10 @@
         <v>358317</v>
       </c>
       <c r="B200">
+        <v>39.292000000000002</v>
+      </c>
+      <c r="C200">
         <v>-123.292</v>
-      </c>
-      <c r="C200">
-        <v>39.292000000000002</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.3">
@@ -4486,10 +4486,10 @@
         <v>358305</v>
       </c>
       <c r="B201">
+        <v>39.292000000000002</v>
+      </c>
+      <c r="C201">
         <v>-123.792</v>
-      </c>
-      <c r="C201">
-        <v>39.292000000000002</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.3">
@@ -4497,10 +4497,10 @@
         <v>358306</v>
       </c>
       <c r="B202">
+        <v>39.292000000000002</v>
+      </c>
+      <c r="C202">
         <v>-123.75</v>
-      </c>
-      <c r="C202">
-        <v>39.292000000000002</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.3">
@@ -4508,10 +4508,10 @@
         <v>358307</v>
       </c>
       <c r="B203">
+        <v>39.292000000000002</v>
+      </c>
+      <c r="C203">
         <v>-123.708</v>
-      </c>
-      <c r="C203">
-        <v>39.292000000000002</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.3">
@@ -4519,10 +4519,10 @@
         <v>358310</v>
       </c>
       <c r="B204">
+        <v>39.292000000000002</v>
+      </c>
+      <c r="C204">
         <v>-123.583</v>
-      </c>
-      <c r="C204">
-        <v>39.292000000000002</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.3">
@@ -4530,10 +4530,10 @@
         <v>358309</v>
       </c>
       <c r="B205">
+        <v>39.292000000000002</v>
+      </c>
+      <c r="C205">
         <v>-123.625</v>
-      </c>
-      <c r="C205">
-        <v>39.292000000000002</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.3">
@@ -4541,10 +4541,10 @@
         <v>358313</v>
       </c>
       <c r="B206">
+        <v>39.292000000000002</v>
+      </c>
+      <c r="C206">
         <v>-123.458</v>
-      </c>
-      <c r="C206">
-        <v>39.292000000000002</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.3">
@@ -4552,10 +4552,10 @@
         <v>358312</v>
       </c>
       <c r="B207">
+        <v>39.292000000000002</v>
+      </c>
+      <c r="C207">
         <v>-123.5</v>
-      </c>
-      <c r="C207">
-        <v>39.292000000000002</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.3">
@@ -4563,10 +4563,10 @@
         <v>358315</v>
       </c>
       <c r="B208">
+        <v>39.292000000000002</v>
+      </c>
+      <c r="C208">
         <v>-123.375</v>
-      </c>
-      <c r="C208">
-        <v>39.292000000000002</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.3">
@@ -4574,10 +4574,10 @@
         <v>358316</v>
       </c>
       <c r="B209">
+        <v>39.292000000000002</v>
+      </c>
+      <c r="C209">
         <v>-123.333</v>
-      </c>
-      <c r="C209">
-        <v>39.292000000000002</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.3">
@@ -4585,10 +4585,10 @@
         <v>356900</v>
       </c>
       <c r="B210">
+        <v>39.332999999999998</v>
+      </c>
+      <c r="C210">
         <v>-123.792</v>
-      </c>
-      <c r="C210">
-        <v>39.332999999999998</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.3">
@@ -4596,10 +4596,10 @@
         <v>356903</v>
       </c>
       <c r="B211">
+        <v>39.332999999999998</v>
+      </c>
+      <c r="C211">
         <v>-123.667</v>
-      </c>
-      <c r="C211">
-        <v>39.332999999999998</v>
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.3">
@@ -4607,10 +4607,10 @@
         <v>356906</v>
       </c>
       <c r="B212">
+        <v>39.332999999999998</v>
+      </c>
+      <c r="C212">
         <v>-123.542</v>
-      </c>
-      <c r="C212">
-        <v>39.332999999999998</v>
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.3">
@@ -4618,10 +4618,10 @@
         <v>356909</v>
       </c>
       <c r="B213">
+        <v>39.332999999999998</v>
+      </c>
+      <c r="C213">
         <v>-123.417</v>
-      </c>
-      <c r="C213">
-        <v>39.332999999999998</v>
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.3">
@@ -4629,10 +4629,10 @@
         <v>356905</v>
       </c>
       <c r="B214">
+        <v>39.332999999999998</v>
+      </c>
+      <c r="C214">
         <v>-123.583</v>
-      </c>
-      <c r="C214">
-        <v>39.332999999999998</v>
       </c>
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.3">
@@ -4640,10 +4640,10 @@
         <v>356901</v>
       </c>
       <c r="B215">
+        <v>39.332999999999998</v>
+      </c>
+      <c r="C215">
         <v>-123.75</v>
-      </c>
-      <c r="C215">
-        <v>39.332999999999998</v>
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.3">
@@ -4651,10 +4651,10 @@
         <v>356902</v>
       </c>
       <c r="B216">
+        <v>39.332999999999998</v>
+      </c>
+      <c r="C216">
         <v>-123.708</v>
-      </c>
-      <c r="C216">
-        <v>39.332999999999998</v>
       </c>
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.3">
@@ -4662,10 +4662,10 @@
         <v>356904</v>
       </c>
       <c r="B217">
+        <v>39.332999999999998</v>
+      </c>
+      <c r="C217">
         <v>-123.625</v>
-      </c>
-      <c r="C217">
-        <v>39.332999999999998</v>
       </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.3">
@@ -4673,10 +4673,10 @@
         <v>356907</v>
       </c>
       <c r="B218">
+        <v>39.332999999999998</v>
+      </c>
+      <c r="C218">
         <v>-123.5</v>
-      </c>
-      <c r="C218">
-        <v>39.332999999999998</v>
       </c>
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.3">
@@ -4684,10 +4684,10 @@
         <v>356908</v>
       </c>
       <c r="B219">
+        <v>39.332999999999998</v>
+      </c>
+      <c r="C219">
         <v>-123.458</v>
-      </c>
-      <c r="C219">
-        <v>39.332999999999998</v>
       </c>
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.3">
@@ -4695,10 +4695,10 @@
         <v>356910</v>
       </c>
       <c r="B220">
+        <v>39.332999999999998</v>
+      </c>
+      <c r="C220">
         <v>-123.375</v>
-      </c>
-      <c r="C220">
-        <v>39.332999999999998</v>
       </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.3">
@@ -4706,10 +4706,10 @@
         <v>356899</v>
       </c>
       <c r="B221">
+        <v>39.332999999999998</v>
+      </c>
+      <c r="C221">
         <v>-123.833</v>
-      </c>
-      <c r="C221">
-        <v>39.332999999999998</v>
       </c>
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.3">
@@ -4717,10 +4717,10 @@
         <v>355501</v>
       </c>
       <c r="B222">
+        <v>39.375</v>
+      </c>
+      <c r="C222">
         <v>-123.542</v>
-      </c>
-      <c r="C222">
-        <v>39.375</v>
       </c>
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.3">
@@ -4728,10 +4728,10 @@
         <v>355500</v>
       </c>
       <c r="B223">
+        <v>39.375</v>
+      </c>
+      <c r="C223">
         <v>-123.583</v>
-      </c>
-      <c r="C223">
-        <v>39.375</v>
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.3">
@@ -4739,10 +4739,10 @@
         <v>355499</v>
       </c>
       <c r="B224">
+        <v>39.375</v>
+      </c>
+      <c r="C224">
         <v>-123.625</v>
-      </c>
-      <c r="C224">
-        <v>39.375</v>
       </c>
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.3">
@@ -4750,10 +4750,10 @@
         <v>355503</v>
       </c>
       <c r="B225">
+        <v>39.375</v>
+      </c>
+      <c r="C225">
         <v>-123.458</v>
-      </c>
-      <c r="C225">
-        <v>39.375</v>
       </c>
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.3">
@@ -4761,10 +4761,10 @@
         <v>355502</v>
       </c>
       <c r="B226">
+        <v>39.375</v>
+      </c>
+      <c r="C226">
         <v>-123.5</v>
-      </c>
-      <c r="C226">
-        <v>39.375</v>
       </c>
     </row>
   </sheetData>
@@ -9169,6 +9169,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100AD1B9453B0FD26428396C40DDB69C7F0" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="7ae69fa2ec7ba05b1cd5ad5facbfed2a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="04ff8bd0-14ef-4472-a603-3a4b6f9fed19" xmlns:ns3="84c16208-172a-4eaa-b33e-1408ce0b909e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="593a7e08a14a0b523a37a1b36e06b6ea" ns2:_="" ns3:_="">
     <xsd:import namespace="04ff8bd0-14ef-4472-a603-3a4b6f9fed19"/>
@@ -9401,15 +9410,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"Blank Document","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="84c16208-172a-4eaa-b33e-1408ce0b909e" xsi:nil="true"/>
@@ -9428,16 +9437,15 @@
 </p:properties>
 </file>
 
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{41E32FE7-C838-46D6-8359-8A7BBC9B619E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3C924A6F-1A37-48C2-B047-4F31E4508879}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9456,19 +9464,19 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{43BD7F1F-596C-48D7-B49B-C059BD9AD9F3}">
   <ds:schemaRefs/>
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06124858-FF52-43B6-9F5F-14F707108C35}">
   <ds:schemaRefs/>
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1A7D180A-E261-4A2D-8CBC-AEEBF9B497B3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
@@ -9485,14 +9493,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{41E32FE7-C838-46D6-8359-8A7BBC9B619E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{0bb6ca0c-ccb3-428b-9d5f-a9c60cad6645}" enabled="1" method="Standard" siteId="{fe186a25-7d49-41e6-9941-05d2281d36c1}" contentBits="0" removed="0"/>

</xml_diff>